<commit_message>
fix: cc_importer corta parseo MAESTRA al detectar segunda tabla
La hoja CC MAESTRA tiene dos tablas. La segunda (Fecha Ingreso CBR)
tenía el mismo nombre de proyectos y sobreescribía los datos correctos
de la primera tabla: entrega, comuna y descuento base quedaban mal.
Ahora el parser se detiene al encontrar el segundo header PROYECTO.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viveprop-platform/data/cc_data.xlsx
+++ b/viveprop-platform/data/cc_data.xlsx
@@ -1127,22 +1127,52 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alto Buzeta</t>
+          <t>Alto Buzeta (MT)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,2%</t>
+          <t>Cerrillos</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>22.22%</t>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Creditú</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>3% 3D</t>
         </is>
       </c>
       <c r="BI9" t="inlineStr"/>
@@ -1160,17 +1190,42 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>27/02/2024</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>Rancagua</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Max 10%</t>
         </is>
       </c>
       <c r="BI10" t="inlineStr"/>
@@ -1183,22 +1238,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jardines de Alvarado</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>15/02/2023</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>0,8%</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>3.21</t>
+          <t>Jardines de Alvarado: solo tipología 3D1B (con descuento máximo de venta de 10%)</t>
         </is>
       </c>
       <c r="BI11" t="inlineStr"/>
@@ -1211,17 +1251,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mirador Mapocho</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>08/05/2024</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Vivienda Social</t>
+          <t>Mirador Mapocho: solo tipología 1D1B (con descuento máximo de venta de 10%)</t>
         </is>
       </c>
       <c r="BI12" t="inlineStr"/>
@@ -1239,17 +1269,42 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>06/07/2023</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>San Joaquín</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2.81</t>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Max 10%</t>
         </is>
       </c>
       <c r="BI13" t="inlineStr"/>
@@ -1267,17 +1322,42 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>03/04/2023</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>La Cisterna</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Max 10%</t>
         </is>
       </c>
       <c r="BI14" t="inlineStr"/>
@@ -1295,17 +1375,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>03/04/2023</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>La Cisterna</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Max 10%</t>
         </is>
       </c>
       <c r="BI15" t="inlineStr"/>
@@ -1318,22 +1423,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Plaza Quilicura</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>24/02/2023</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>0,8%</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>3.18</t>
+          <t>Plaza Quilicura: Se deben vender todos los departamentos con estacionamiento de manera obligatoria; Estacionamientos bajan a UF 250 (Precio anterior UF 290)</t>
         </is>
       </c>
       <c r="BI16" t="inlineStr"/>
@@ -1351,17 +1441,42 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>31/12/2021</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>La Cisterna</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4.33</t>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Max 10%</t>
         </is>
       </c>
       <c r="BI17" t="inlineStr"/>
@@ -1374,22 +1489,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vista Costanera</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>14/09/2022</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>0,8%</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>3.62</t>
+          <t>Vista Costanera: Bajan los estacionamientos a 2 x UF 500</t>
         </is>
       </c>
       <c r="BI18" t="inlineStr"/>
@@ -1407,17 +1507,47 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>26/11/2024</t>
+          <t>Inmediata</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,2%</t>
+          <t>Puerto Montt</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>GOP</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Max 10%</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2% 3D</t>
         </is>
       </c>
       <c r="BI19" t="inlineStr"/>

</xml_diff>